<commit_message>
Sync backend test count after the rmse fix
</commit_message>
<xml_diff>
--- a/TEST_CASES_new.xlsx
+++ b/TEST_CASES_new.xlsx
@@ -7330,6 +7330,7 @@
         <v>51</v>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -7359,10 +7360,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C18" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -7396,10 +7397,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C20" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
List every test file and count the uncollectable tests
</commit_message>
<xml_diff>
--- a/TEST_CASES_new.xlsx
+++ b/TEST_CASES_new.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$J$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$J$146</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J145"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5854,7 +5854,7 @@
       <c r="G116" s="3" t="inlineStr"/>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>test_planegrid.py</t>
+          <t>backend/tests/test_planegrid.py</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
@@ -5890,7 +5890,7 @@
       <c r="G117" s="3" t="inlineStr"/>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>test_planegrid.py</t>
+          <t>backend/tests/test_planegrid.py</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -5926,7 +5926,7 @@
       <c r="G118" s="3" t="inlineStr"/>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>test_planegrid.py</t>
+          <t>backend/tests/test_planegrid.py</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
@@ -5962,7 +5962,7 @@
       <c r="G119" s="3" t="inlineStr"/>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>test_planegrid.py</t>
+          <t>backend/tests/test_planegrid.py</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">
@@ -5998,7 +5998,7 @@
       <c r="G120" s="3" t="inlineStr"/>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>test_planegrid.py</t>
+          <t>backend/tests/test_planegrid.py</t>
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr">
@@ -6034,7 +6034,7 @@
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>test_config.py</t>
+          <t>backend/tests/test_config.py</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr">
@@ -6070,7 +6070,7 @@
       <c r="G122" s="3" t="inlineStr"/>
       <c r="H122" s="3" t="inlineStr">
         <is>
-          <t>test_models.py</t>
+          <t>backend/tests/test_models.py</t>
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr">
@@ -6106,7 +6106,7 @@
       <c r="G123" s="3" t="inlineStr"/>
       <c r="H123" s="3" t="inlineStr">
         <is>
-          <t>test_auth.py</t>
+          <t>backend/tests/test_auth.py</t>
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr">
@@ -6142,7 +6142,7 @@
       <c r="G124" s="3" t="inlineStr"/>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>lib/api.test.js</t>
+          <t>frontend/src/lib/api.test.js</t>
         </is>
       </c>
       <c r="I124" s="2" t="inlineStr">
@@ -6178,7 +6178,7 @@
       <c r="G125" s="3" t="inlineStr"/>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>lib/api.test.js</t>
+          <t>frontend/src/lib/api.test.js</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr">
@@ -6214,7 +6214,7 @@
       <c r="G126" s="3" t="inlineStr"/>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>components/ApiErrorBanner.test.jsx</t>
+          <t>frontend/src/components/ApiErrorBanner.test.jsx</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       <c r="G127" s="3" t="inlineStr"/>
       <c r="H127" s="3" t="inlineStr">
         <is>
-          <t>components/RequireAuth.test.jsx</t>
+          <t>frontend/src/components/RequireAuth.test.jsx</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr">
@@ -6908,8 +6908,44 @@
       </c>
       <c r="J145" s="2" t="inlineStr"/>
     </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Automated Unit Tests (รันอัตโนมัติอยู่แล้ว)</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>🟢 BE-23</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>floorcalib — homography จากจุด 4 ตัวขึ้น, จุด collinear ถูกปฏิเสธ, project/invert round-trip, rmse สะท้อน noise, save/load</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr"/>
+      <c r="F146" s="3" t="inlineStr"/>
+      <c r="G146" s="3" t="inlineStr"/>
+      <c r="H146" s="3" t="inlineStr">
+        <is>
+          <t>backend/tests/test_floorcalib.py</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J145"/>
+  <autoFilter ref="A1:J146"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7232,16 +7268,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -7312,16 +7348,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C15" t="n">
         <v>114</v>
       </c>
       <c r="D15" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E15" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -7370,7 +7406,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>test_models.py / test_auth.py: ต้องมี sqlalchemy ซึ่งไม่ได้ติดตั้งบนเครื่องนี้ จึงไม่นับ</t>
+          <t>test_auth.py (11) และ test_models.py (5) รวม 16 เทสต์ รันบนเครื่องนี้ไม่ได้ เพราะไม่มี sqlalchemy/httpx จึงไม่นับใน 133</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record observed manual results and recompute the summary
</commit_message>
<xml_diff>
--- a/TEST_CASES_new.xlsx
+++ b/TEST_CASES_new.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:K146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -521,6 +521,11 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Observed Result</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -568,7 +573,12 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>login 200 + access_token</t>
+          <t>POST /api/auth/login</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>HTTP 200 · token 203 chars · username=qa_manual_2026</t>
         </is>
       </c>
     </row>
@@ -618,7 +628,12 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>401 Invalid credentials</t>
+          <t>รหัสผิด</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>HTTP 401 · Invalid credentials</t>
         </is>
       </c>
     </row>
@@ -668,7 +683,12 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>user ไม่มีในระบบ</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>HTTP 401 · Invalid credentials</t>
         </is>
       </c>
     </row>
@@ -713,12 +733,17 @@
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Needs Browser</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>UI redirect (RequireAuth)</t>
+          <t>GET /api/auth/me ไม่มี token</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>HTTP 401</t>
         </is>
       </c>
     </row>
@@ -767,7 +792,12 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>expired token -&gt; 401</t>
+          <t>JWT exp=1500000001 หมดอายุ</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>HTTP 401</t>
         </is>
       </c>
     </row>
@@ -816,7 +846,12 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>bad token -&gt; 401</t>
+          <t>token ไม่ใช่ JWT</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>HTTP 401</t>
         </is>
       </c>
     </row>
@@ -865,7 +900,12 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>no header -&gt; 401</t>
+          <t>ไม่มี Authorization header</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>HTTP 401</t>
         </is>
       </c>
     </row>
@@ -914,7 +954,12 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>/me 200 + {id, username}</t>
+          <t>token ที่ถูกต้อง</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>HTTP 200 · username=qa_manual_2026</t>
         </is>
       </c>
     </row>
@@ -963,7 +1008,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>no token -&gt; 401</t>
+          <t>POST /api/auth/register ไม่มี token</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>HTTP 401</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1062,12 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>username 1 char -&gt; 400</t>
+          <t>ชื่อ 'a'</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>HTTP 400 · Username must be at least 2 characters</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1116,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>password 1 char -&gt; 400</t>
+          <t>รหัส 'ab'</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>HTTP 400 · Password must be at least 4 characters</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1171,12 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>dup admin -&gt; 409</t>
+          <t>ชื่อซ้ำ</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>HTTP 409 · Username already exists</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1225,12 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>register 200 + token</t>
+          <t>register ด้วย token</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>HTTP 200 · สร้าง qa_manual_created_1 สำเร็จ</t>
         </is>
       </c>
     </row>
@@ -1205,12 +1275,17 @@
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Needs Browser</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>UI logout button</t>
+          <t>GET /api/settings ด้วย token เสีย</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>HTTP 401</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1335,12 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>covered by FE-01 auto</t>
+          <t>ดู header จริงตอนเปิด /dashboard</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Authorization: Bearer ติดไปกับ request ของแอปเอง</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1539,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>covered by FE-02 auto (401 redirect)</t>
+          <t>evidence/API-05_invalid_token_redirects_login.png</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>เด้งจาก /dobot ไป /login เมื่อ token เสีย</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1593,12 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>covered by FE-02 auto</t>
+          <t>ทดสอบขณะล็อกอินอยู่แล้ว</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>401 จาก /api/auth/login · ยังอยู่ /dashboard ไม่เด้ง</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1696,12 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>status 200, robot connected=True</t>
+          <t>evidence/DASH-01_dashboard.png</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>connected=true · robot_mode_label=RUNNING · camera_running=true · IP 192.168.10.110</t>
         </is>
       </c>
     </row>
@@ -3364,12 +3459,17 @@
       <c r="H59" s="3" t="inlineStr"/>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Needs Browser</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>UI tab</t>
+          <t>evidence/TP-01_tab_*.png</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>แท็บ Align/Jog/Grid/Draw มีครบ · สลับแต่ละแท็บแล้ว class active ถูกต้อง</t>
         </is>
       </c>
     </row>
@@ -3464,12 +3564,17 @@
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Needs Browser</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>UI pills</t>
+          <t>evidence/TP-05_grid_tab.png</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>pill: Connected · Camera 1 — offline · 4/4 marked · grid 2x2 Z=148.6mm span=202.6mm rmse=0.2447mm · 0/5 recorded</t>
         </is>
       </c>
     </row>
@@ -3514,12 +3619,17 @@
       <c r="H62" s="3" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Needs Browser</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>UI quick actions</t>
+          <t>evidence/TP-05_grid_tab.png</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>quick actions: Clear Error / Init / Home / Set Grid / Reset Grid / Reset test points</t>
         </is>
       </c>
     </row>
@@ -3564,12 +3674,17 @@
       <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Needs Browser</t>
+          <t>Pass (observed)</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>UI grid setup</t>
+          <t>evidence/TP-05_grid_tab.png</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>GRID SETUP (2×2) · ช่อง ROWS/COLS = 2, min=2 max=7 · ไม่ได้เปลี่ยนค่าเพราะการเปลี่ยนขนาดจะล้าง mark เดิม</t>
         </is>
       </c>
     </row>
@@ -3614,10 +3729,19 @@
       <c r="H64" s="3" t="inlineStr"/>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Needs Browser</t>
-        </is>
-      </c>
-      <c r="J64" s="2" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>evidence/TP-05_grid_tab.png</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>cells matrix = R1C1, R1C2, R2C1, R2C2 ตรงกับ grid 2×2</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3801,10 +3925,19 @@
       <c r="H68" s="3" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Needs Browser</t>
-        </is>
-      </c>
-      <c r="J68" s="2" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>evidence/TP-01_tab_Align.png</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>COORDINATE FRAME: Tool / User / Apply อยู่ในแท็บ Align</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4758,7 +4891,12 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>no token -&gt; 401</t>
+          <t>evidence/HTTP_sec_transcript.json</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ไม่มี token→401 · token เสีย→401 · token ถูกต้อง→200 · สแกน 8 GET endpoint ไม่มีตัวไหนตอบ 200 โดยไม่มี token</t>
         </is>
       </c>
     </row>
@@ -4808,7 +4946,12 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>evil origin -&gt; ACAO none</t>
+          <t>ALLOWED_ORIGINS=http://localhost:5173,http://127.0.0.1,http://192.168.10.104</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ACAO ตรงกับ origin ที่อนุญาต 3 ตัว · evil.example.com ไม่ได้ ACAO</t>
         </is>
       </c>
     </row>
@@ -4857,7 +5000,12 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>OPTIONS -&gt; 405 (ไม่โดน 401)</t>
+          <t>OPTIONS /api/map/status</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>HTTP 200 (ไม่ใช่ 401)</t>
         </is>
       </c>
     </row>
@@ -4906,7 +5054,12 @@
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>backend root 200 message; หลัง nginx / = SPA (ปกติ)</t>
+          <t>GET /</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>HTTP 200 · Robot Arm API is running</t>
         </is>
       </c>
     </row>
@@ -5679,6 +5832,21 @@
           <t>เห็น events (robot/camera/align/scan) พร้อม user</t>
         </is>
       </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>evidence/LOG-01_activity_log.png</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>100 รายการ ครบ 5 คอลัมน์ (เวลา/ผู้ใช้/อุปกรณ์/การกระทำ/รายละเอียด)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5714,6 +5882,21 @@
       <c r="G112" t="inlineStr">
         <is>
           <t>ผลกรองถูกต้อง (GET /api/devices/events)</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>evidence/LOG-02_filter_estop.png</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>filter robot→เหลือ ROBOT · filter estop→TESTOP · ค้น 'strokes'→เจอ 4 รายการ DRAW · รีเซ็ตกลับได้ครบ</t>
         </is>
       </c>
     </row>
@@ -6956,7 +7139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7027,13 +7210,18 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 14/14</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -7060,6 +7248,11 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 3/7</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7085,6 +7278,11 @@
       <c r="G4" t="n">
         <v>1</v>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 1/2</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7110,6 +7308,11 @@
       <c r="G5" t="n">
         <v>10</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 0/4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7135,6 +7338,11 @@
       <c r="G6" t="n">
         <v>7</v>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 0/7</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7152,13 +7360,18 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>23</v>
+        <v>17</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 6/6</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -7185,6 +7398,11 @@
       <c r="G8" t="n">
         <v>8</v>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 0/1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7210,6 +7428,11 @@
       <c r="G9" t="n">
         <v>4</v>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 0/1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7235,6 +7458,11 @@
       <c r="G10" t="n">
         <v>5</v>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 0/4</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7260,6 +7488,11 @@
       <c r="G11" t="n">
         <v>0</v>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 4/4</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7315,6 +7548,11 @@
       <c r="G13" t="n">
         <v>6</v>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 0/3</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7332,13 +7570,18 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 2/2</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -7357,13 +7600,18 @@
         <v>31</v>
       </c>
       <c r="E15" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>51</v>
+        <v>59</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>manual 55 pass (มีหลักฐาน 30) + automated 31 pass · blocked 59</t>
+        </is>
       </c>
     </row>
     <row r="16"/>
@@ -7440,6 +7688,59 @@
       </c>
       <c r="D20" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MANUAL TEST RUN (2026-10-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>รันด้วย automation ต่อระบบจริง</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>30</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>AUTH 14 · SEC 4 · API 3 · DASH-01 · LOG 2 · TP 6 — หลักฐานใน evidence/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>บันทึก Pass จากเซสชันก่อน</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>25</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ไม่ได้วัดรอบนี้ — ไม่มีค่าที่สังเกตได้</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ยังไม่ได้ทำ (รอเงื่อนไข/หน้าเครื่อง)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>59</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>คู่มือ: MANUAL_TESTS_ON_SITE.md</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Verify the public tunnel and log the align WebSocket failure
</commit_message>
<xml_diff>
--- a/TEST_CASES_new.xlsx
+++ b/TEST_CASES_new.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$J$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$J$151</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K146"/>
+  <dimension ref="A1:K151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7127,8 +7127,233 @@
       </c>
       <c r="J146" s="2" t="inlineStr"/>
     </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Public Access (Cloudflare Tunnel)</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>🔵 PUB-01</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>HTTPS public URL เปิดได้และโหลด SPA</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr"/>
+      <c r="F147" s="3" t="inlineStr"/>
+      <c r="G147" s="3" t="inlineStr"/>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>ทดสอบผ่าน https://robot-web.box-dex.win</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>เทียบ LAN: build เดียวกัน (index-D1q7yGYr.js)</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>HTTP 200 · title=frontend · bundle index-D1q7yGYr.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Public Access (Cloudflare Tunnel)</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>🔵 PUB-02</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>login ผ่าน tunnel</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr"/>
+      <c r="F148" s="3" t="inlineStr"/>
+      <c r="G148" s="3" t="inlineStr"/>
+      <c r="H148" s="3" t="inlineStr">
+        <is>
+          <t>ทดสอบผ่าน https://robot-web.box-dex.win</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>qa_manual_2026</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>HTTP 200 · ได้ access_token</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Public Access (Cloudflare Tunnel)</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>🔵 PUB-03</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>auth ผ่าน tunnel</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr"/>
+      <c r="F149" s="3" t="inlineStr"/>
+      <c r="G149" s="3" t="inlineStr"/>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>ทดสอบผ่าน https://robot-web.box-dex.win</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>ตรวจแล้วไม่มีช่องโหว่เหมือนกับ LAN</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>มี token→200 · ไม่มี token→401</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Public Access (Cloudflare Tunnel)</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>🔵 PUB-04</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>WebSocket /ws/joints ผ่าน tunnel</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr"/>
+      <c r="F150" s="3" t="inlineStr"/>
+      <c r="G150" s="3" t="inlineStr"/>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>ทดสอบผ่าน https://robot-web.box-dex.win</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>tunnel ส่ง Upgrade header ได้ถูกต้อง</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>wss handshake → 101 Switching Protocols</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>Public Access (Cloudflare Tunnel)</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>🔵 PUB-05</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>WebSocket /api/scan/ws/align ผ่าน tunnel</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr"/>
+      <c r="F151" s="3" t="inlineStr"/>
+      <c r="G151" s="3" t="inlineStr"/>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>ทดสอบผ่าน https://robot-web.box-dex.win</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>ยืนยันว่าเป็นบั๊กฝั่ง backend ไม่ใช่ Cloudflare · middleware บล็อก /api/* และ deployed build ไม่มี route นี้</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>wss handshake → 401 Unauthorized (เหมือน LAN)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J146"/>
+  <autoFilter ref="A1:J151"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7139,7 +7364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7497,247 +7722,277 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Automated Unit Tests (รันอัตโนมัติอยู่แล้ว)</t>
+          <t>Public Access (Cloudflare Tunnel)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="n">
-        <v>31</v>
-      </c>
       <c r="E12" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>เพิ่มรายการ automated ของ session ล่าสุด</t>
+          <t>ตรวจผ่าน Cloudflare Tunnel</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Scan &amp; Fuse (/scan panel)</t>
+          <t>Automated Unit Tests (รันอัตโนมัติอยู่แล้ว)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>มีหลักฐานรอบนี้ 0/3</t>
+          <t>เพิ่มรายการ automated ของ session ล่าสุด</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Activity Log (/logs)</t>
+          <t>Scan &amp; Fuse (/scan panel)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>มีหลักฐานรอบนี้ 2/2</t>
+          <t>มีหลักฐานรอบนี้ 0/3</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TOTAL (test cases)</t>
+          <t>Activity Log (/logs)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>145</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>114</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>86</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>มีหลักฐานรอบนี้ 2/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TOTAL (test cases)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>150</v>
+      </c>
+      <c r="C16" t="n">
+        <v>119</v>
+      </c>
+      <c r="D16" t="n">
+        <v>31</v>
+      </c>
+      <c r="E16" t="n">
+        <v>90</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
         <v>59</v>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>manual 55 pass (มีหลักฐาน 30) + automated 31 pass · blocked 59</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Automated test run (latest)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-    </row>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>manual 119 = pass 59 + fail 1 + blocked 59 · automated 31 pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Backend pytest (backend/tests)</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>133</v>
-      </c>
-      <c r="C18" t="n">
-        <v>133</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>test_auth.py (11) และ test_models.py (5) รวม 16 เทสต์ รันบนเครื่องนี้ไม่ได้ เพราะไม่มี sqlalchemy/httpx จึงไม่นับใน 133</t>
+          <t>Automated test run (latest)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Frontend vitest (frontend/src)</t>
+          <t>Backend pytest (backend/tests)</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>87</v>
+        <v>133</v>
       </c>
       <c r="C19" t="n">
-        <v>87</v>
+        <v>133</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>test_auth.py (11) และ test_models.py (5) รวม 16 เทสต์ รันบนเครื่องนี้ไม่ได้ เพราะไม่มี sqlalchemy/httpx จึงไม่นับใน 133</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL tests</t>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Frontend vitest (frontend/src)</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>220</v>
+        <v>87</v>
       </c>
       <c r="C20" t="n">
-        <v>220</v>
+        <v>87</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>MANUAL TEST RUN (2026-10-06)</t>
-        </is>
-      </c>
-    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL tests</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>220</v>
+      </c>
+      <c r="C21" t="n">
+        <v>220</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>รันด้วย automation ต่อระบบจริง</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>30</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>AUTH 14 · SEC 4 · API 3 · DASH-01 · LOG 2 · TP 6 — หลักฐานใน evidence/</t>
+          <t>MANUAL TEST RUN (2026-10-06)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>บันทึก Pass จากเซสชันก่อน</t>
+          <t>รันด้วย automation ต่อระบบจริง</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>ไม่ได้วัดรอบนี้ — ไม่มีค่าที่สังเกตได้</t>
+          <t>AUTH 14 · SEC 4 · API 3 · DASH-01 · LOG 2 · TP 6 · PUB 5 — หลักฐานใน evidence/</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>บันทึก Pass จากเซสชันก่อน</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ไม่ได้วัดรอบนี้ — ไม่มีค่าที่สังเกตได้</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>ยังไม่ได้ทำ (รอเงื่อนไข/หน้าเครื่อง)</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B26" t="n">
         <v>59</v>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>คู่มือ: MANUAL_TESTS_ON_SITE.md</t>
         </is>

</xml_diff>

<commit_message>
Forward websocket upgrades for the scan endpoints through nginx
</commit_message>
<xml_diff>
--- a/TEST_CASES_new.xlsx
+++ b/TEST_CASES_new.xlsx
@@ -7338,17 +7338,17 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
         <is>
-          <t>ยืนยันว่าเป็นบั๊กฝั่ง backend ไม่ใช่ Cloudflare · middleware บล็อก /api/* และ deployed build ไม่มี route นี้</t>
+          <t>แก้แล้ว: middleware ข้าม websocket handshake + nginx ส่ง Upgrade ที่ /api/scan/ws · console error 0</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>wss handshake → 401 Unauthorized (เหมือน LAN)</t>
+          <t>wss handshake → 101 Switching Protocols (ผ่าน Cloudflare / nginx / ตรง :8000 ครบทั้ง 3 ทาง)</t>
         </is>
       </c>
     </row>
@@ -7735,10 +7735,10 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -7855,17 +7855,17 @@
         <v>31</v>
       </c>
       <c r="E16" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>59</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>manual 119 = pass 59 + fail 1 + blocked 59 · automated 31 pass</t>
+          <t>manual 119 = pass 60 + fail 0 + blocked 59 · automated 31 pass</t>
         </is>
       </c>
     </row>

</xml_diff>